<commit_message>
Add vaccination policy scenarios and update related configurations
- Updated `.gitignore` to include new vaccination policy scenario results for 2Xvax and 4Xvax.
- Adjusted `mpox2024_parameters.m` to read additional file paths for vaccination transition data.
- Enhanced `mpox2024_shellMod.m` to support dynamic selection of vaccination transition paths based on the enabled vaccination policy.
- Updated `Mpox2024_ShellScript.m` to reflect changes in scenario configurations and added vaccination policy settings.
</commit_message>
<xml_diff>
--- a/input/Inputs_mpox2024_set2.xlsx
+++ b/input/Inputs_mpox2024_set2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liangshiting/Desktop/USCResearch/Mpox_2024/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liangshiting/Desktop/USCResearch/Mpox_2024/Code_updated/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB3E1A94-F93C-B141-9CDD-D5956B27EA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5FC8264-D882-0B4B-A10A-E104C705FF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{0FC07F83-73B4-4DAF-8E73-97E4E92D674F}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" firstSheet="6" activeTab="18" xr2:uid="{0FC07F83-73B4-4DAF-8E73-97E4E92D674F}"/>
   </bookViews>
   <sheets>
     <sheet name="SimDuration" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="319">
   <si>
     <t>Birth Dynamics</t>
   </si>
@@ -1000,6 +1000,18 @@
   </si>
   <si>
     <t>../input/vac_1_wk9_half.csv</t>
+  </si>
+  <si>
+    <t>../input/vac_1_new2_2X.csv</t>
+  </si>
+  <si>
+    <t>2X vax</t>
+  </si>
+  <si>
+    <t>4X vax</t>
+  </si>
+  <si>
+    <t>../input/vac_1_new2_4X.csv</t>
   </si>
 </sst>
 </file>
@@ -3627,7 +3639,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CCBAD9-D596-4993-A838-C32E90D12062}">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.6640625" bestFit="1" customWidth="1"/>
@@ -4097,6 +4109,22 @@
       </c>
       <c r="B58" s="33" t="s">
         <v>314</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>316</v>
+      </c>
+      <c r="B59" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>317</v>
+      </c>
+      <c r="B60" t="s">
+        <v>318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 10X vax policy scenarios
</commit_message>
<xml_diff>
--- a/input/Inputs_mpox2024_set2.xlsx
+++ b/input/Inputs_mpox2024_set2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liangshiting/Desktop/USCResearch/Mpox_2024/Code_updated/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5FC8264-D882-0B4B-A10A-E104C705FF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C326E825-02F9-3D4C-A316-EC7876B03289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" firstSheet="6" activeTab="18" xr2:uid="{0FC07F83-73B4-4DAF-8E73-97E4E92D674F}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="321">
   <si>
     <t>Birth Dynamics</t>
   </si>
@@ -1012,6 +1012,12 @@
   </si>
   <si>
     <t>../input/vac_1_new2_4X.csv</t>
+  </si>
+  <si>
+    <t>10X vax</t>
+  </si>
+  <si>
+    <t>../input/vac_1_new2_10X.csv</t>
   </si>
 </sst>
 </file>
@@ -3639,7 +3645,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2CCBAD9-D596-4993-A838-C32E90D12062}">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.6640625" bestFit="1" customWidth="1"/>
@@ -4125,6 +4131,14 @@
       </c>
       <c r="B60" t="s">
         <v>318</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>319</v>
+      </c>
+      <c r="B61" t="s">
+        <v>320</v>
       </c>
     </row>
   </sheetData>

</xml_diff>